<commit_message>
Replace flag_gompertz with flag_model
</commit_message>
<xml_diff>
--- a/inst/extdata/example_metadata.xlsx
+++ b/inst/extdata/example_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Arlan\Desktop\rumenGP\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7108E426-DBFB-4CB9-A718-F0BF6FF4E937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67741837-2DB4-44E1-B940-DBDAE8BDF2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{13B5C980-F356-944D-8F6C-78B1F36B7411}"/>
   </bookViews>
@@ -41,9 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="10">
   <si>
-    <t>Sample</t>
-  </si>
-  <si>
     <t>Bottle</t>
   </si>
   <si>
@@ -69,6 +66,9 @@
   </si>
   <si>
     <t>Plant_C</t>
+  </si>
+  <si>
+    <t>Treatment</t>
   </si>
 </sst>
 </file>
@@ -471,19 +471,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -497,7 +497,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E2" s="2">
         <v>6.24</v>
@@ -514,7 +514,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E3" s="2">
         <v>6.22</v>
@@ -531,7 +531,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" s="2">
         <v>6.24</v>
@@ -548,7 +548,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" s="2">
         <v>6.3</v>
@@ -565,7 +565,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" s="2">
         <v>6.15</v>
@@ -582,7 +582,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" s="2">
         <v>6.16</v>
@@ -599,7 +599,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="2">
         <v>6.13</v>
@@ -616,7 +616,7 @@
         <v>2</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" s="2">
         <v>6.12</v>
@@ -633,7 +633,7 @@
         <v>3</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="2">
         <v>6.12</v>
@@ -650,7 +650,7 @@
         <v>4</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="2">
         <v>6.26</v>
@@ -667,7 +667,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12" s="2">
         <v>6.12</v>
@@ -684,7 +684,7 @@
         <v>6</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="2">
         <v>6.17</v>
@@ -701,7 +701,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E14" s="2">
         <v>6.15</v>
@@ -718,7 +718,7 @@
         <v>2</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E15" s="2">
         <v>6.17</v>
@@ -735,7 +735,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E16" s="2">
         <v>6.12</v>
@@ -752,7 +752,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E17" s="2">
         <v>6.25</v>
@@ -769,7 +769,7 @@
         <v>5</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E18" s="2">
         <v>6.12</v>
@@ -786,7 +786,7 @@
         <v>6</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="2">
         <v>6.08</v>
@@ -803,7 +803,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="2">
         <v>6.1</v>
@@ -820,7 +820,7 @@
         <v>2</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E21" s="2">
         <v>6.17</v>
@@ -837,7 +837,7 @@
         <v>3</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" s="2">
         <v>6.16</v>
@@ -854,7 +854,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23" s="2">
         <v>6.58</v>
@@ -871,7 +871,7 @@
         <v>2</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E24" s="2">
         <v>6.84</v>
@@ -888,7 +888,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" s="2">
         <v>6.53</v>

</xml_diff>